<commit_message>
Fix two Thai-language extraction bugs found by running the samples
Both were regex mistakes that unit tests never reached, and both produced
wrong output on 03-standup-th.txt:

- readMeta split the attendee list on [,、และ]. "และ" in a character class is
  three separate characters, so the ล inside "พลอย" was a delimiter: three
  Thai attendees came out as six entries including "พ", "อย" and "อรรถพ".
  Split on the word instead.

- The owner pattern for ฝาก / มอบหมายให้ captured `คุณ?`, which makes only the
  ณ optional — so it matched "คุณสมชาย" but never a bare Thai name. "ฝาก
  อรรถพล ช่วยเช็ค config" lost its owner and was reported as unowned.

Three regression tests, one per behaviour plus the honorific case that already
worked, so neither pattern can quietly revert.

Documents regenerated (34 unit cases). CLAUDE.md and the README revision log
gain the note that regenerating always restamps an embedded timestamp, so the
files show as modified even when the content is identical.
</commit_message>
<xml_diff>
--- a/docs/generated/Unit-Test-Cases.xlsx
+++ b/docs/generated/Unit-Test-Cases.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="192">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -170,6 +170,21 @@
     <t>UT-009</t>
   </si>
   <si>
+    <t>splits a Thai attendee list on the word และ, not on its letters</t>
+  </si>
+  <si>
+    <t>The system splits a Thai attendee list on the word และ, not on its letters.</t>
+  </si>
+  <si>
+    <t>"และ" is a word. As a character class it split "พลอย" into "พ" and "อย".</t>
+  </si>
+  <si>
+    <t>backend/tests/parse.test.ts:56</t>
+  </si>
+  <si>
+    <t>UT-010</t>
+  </si>
+  <si>
     <t>includes a listed attendee who never speaks</t>
   </si>
   <si>
@@ -179,10 +194,10 @@
     <t>A Participant need not be a Speaker — see CONTEXT.md.</t>
   </si>
   <si>
-    <t>backend/tests/parse.test.ts:56</t>
-  </si>
-  <si>
-    <t>UT-010</t>
+    <t>backend/tests/parse.test.ts:64</t>
+  </si>
+  <si>
+    <t>UT-011</t>
   </si>
   <si>
     <t>Distill (backend/src/distill.ts)</t>
@@ -203,7 +218,7 @@
     <t>backend/tests/distill.test.ts:12</t>
   </si>
   <si>
-    <t>UT-011</t>
+    <t>UT-012</t>
   </si>
   <si>
     <t>opens one topic per cue even when the transcript carries a header block</t>
@@ -218,7 +233,7 @@
     <t>backend/tests/distill.test.ts:20</t>
   </si>
   <si>
-    <t>UT-012</t>
+    <t>UT-013</t>
   </si>
   <si>
     <t>attributes an action item to the named owner</t>
@@ -230,7 +245,7 @@
     <t>backend/tests/distill.test.ts:35</t>
   </si>
   <si>
-    <t>UT-013</t>
+    <t>UT-014</t>
   </si>
   <si>
     <t>attributes a self-assignment to the speaker</t>
@@ -242,7 +257,7 @@
     <t>backend/tests/distill.test.ts:42</t>
   </si>
   <si>
-    <t>UT-014</t>
+    <t>UT-015</t>
   </si>
   <si>
     <t>leaves the owner null rather than guessing</t>
@@ -257,7 +272,34 @@
     <t>backend/tests/distill.test.ts:48</t>
   </si>
   <si>
-    <t>UT-015</t>
+    <t>UT-016</t>
+  </si>
+  <si>
+    <t>attributes a Thai ฝาก assignment to the name that follows it</t>
+  </si>
+  <si>
+    <t>The system attributes a Thai ฝาก assignment to the name that follows it.</t>
+  </si>
+  <si>
+    <t>`คุณ?` made only the ณ optional, so an unprefixed Thai name was never captured.</t>
+  </si>
+  <si>
+    <t>backend/tests/distill.test.ts:54</t>
+  </si>
+  <si>
+    <t>UT-017</t>
+  </si>
+  <si>
+    <t>keeps the honorific when the transcript wrote one</t>
+  </si>
+  <si>
+    <t>The system keeps the honorific when the transcript wrote one.</t>
+  </si>
+  <si>
+    <t>backend/tests/distill.test.ts:59</t>
+  </si>
+  <si>
+    <t>UT-018</t>
   </si>
   <si>
     <t>keeps a vague deadline as raw text and refuses to resolve it to a date</t>
@@ -266,10 +308,10 @@
     <t>The system keeps a vague deadline as raw text and refuses to resolve it to a date.</t>
   </si>
   <si>
-    <t>backend/tests/distill.test.ts:53</t>
-  </si>
-  <si>
-    <t>UT-016</t>
+    <t>backend/tests/distill.test.ts:64</t>
+  </si>
+  <si>
+    <t>UT-019</t>
   </si>
   <si>
     <t>records a go-live as a milestone</t>
@@ -278,10 +320,10 @@
     <t>The system records a go-live as a milestone.</t>
   </si>
   <si>
-    <t>backend/tests/distill.test.ts:60</t>
-  </si>
-  <si>
-    <t>UT-017</t>
+    <t>backend/tests/distill.test.ts:71</t>
+  </si>
+  <si>
+    <t>UT-020</t>
   </si>
   <si>
     <t>handles a Thai transcript</t>
@@ -290,10 +332,10 @@
     <t>The system handles a Thai transcript.</t>
   </si>
   <si>
-    <t>backend/tests/distill.test.ts:65</t>
-  </si>
-  <si>
-    <t>UT-018</t>
+    <t>backend/tests/distill.test.ts:76</t>
+  </si>
+  <si>
+    <t>UT-021</t>
   </si>
   <si>
     <t>Analyze (backend/src/analyze.ts)</t>
@@ -317,7 +359,7 @@
     <t>backend/tests/analyze.test.ts:9</t>
   </si>
   <si>
-    <t>UT-019</t>
+    <t>UT-022</t>
   </si>
   <si>
     <t>does not flag a meeting where any topic reached a decision</t>
@@ -329,7 +371,7 @@
     <t>backend/tests/analyze.test.ts:14</t>
   </si>
   <si>
-    <t>UT-020</t>
+    <t>UT-023</t>
   </si>
   <si>
     <t>ownership</t>
@@ -347,7 +389,7 @@
     <t>backend/tests/analyze.test.ts:22</t>
   </si>
   <si>
-    <t>UT-021</t>
+    <t>UT-024</t>
   </si>
   <si>
     <t>flags look-alike owner names across different meetings</t>
@@ -359,7 +401,7 @@
     <t>backend/tests/analyze.test.ts:28</t>
   </si>
   <si>
-    <t>UT-022</t>
+    <t>UT-025</t>
   </si>
   <si>
     <t>does not flag two genuinely different owners</t>
@@ -371,7 +413,7 @@
     <t>backend/tests/analyze.test.ts:35</t>
   </si>
   <si>
-    <t>UT-023</t>
+    <t>UT-026</t>
   </si>
   <si>
     <t>strips honorifics and casing only for comparison</t>
@@ -383,7 +425,7 @@
     <t>backend/tests/analyze.test.ts:42</t>
   </si>
   <si>
-    <t>UT-024</t>
+    <t>UT-027</t>
   </si>
   <si>
     <t>date problems</t>
@@ -401,7 +443,7 @@
     <t>backend/tests/analyze.test.ts:49</t>
   </si>
   <si>
-    <t>UT-025</t>
+    <t>UT-028</t>
   </si>
   <si>
     <t>does not flag an action item that mentioned no deadline at all</t>
@@ -413,7 +455,7 @@
     <t>backend/tests/analyze.test.ts:56</t>
   </si>
   <si>
-    <t>UT-026</t>
+    <t>UT-029</t>
   </si>
   <si>
     <t>flags an action item due after a milestone it should precede</t>
@@ -428,7 +470,7 @@
     <t>backend/tests/analyze.test.ts:62</t>
   </si>
   <si>
-    <t>UT-027</t>
+    <t>UT-030</t>
   </si>
   <si>
     <t>flags a deadline that falls before the meeting itself</t>
@@ -440,7 +482,7 @@
     <t>backend/tests/analyze.test.ts:71</t>
   </si>
   <si>
-    <t>UT-028</t>
+    <t>UT-031</t>
   </si>
   <si>
     <t>leaves a deadline comfortably before the milestone alone</t>
@@ -452,7 +494,7 @@
     <t>backend/tests/analyze.test.ts:79</t>
   </si>
   <si>
-    <t>UT-029</t>
+    <t>UT-032</t>
   </si>
   <si>
     <t>Rollup (backend/src/rollup.ts)</t>
@@ -473,7 +515,7 @@
     <t>backend/tests/rollup.test.ts:6</t>
   </si>
   <si>
-    <t>UT-030</t>
+    <t>UT-033</t>
   </si>
   <si>
     <t>keeps look-alike owner names in separate groups</t>
@@ -488,7 +530,7 @@
     <t>backend/tests/rollup.test.ts:16</t>
   </si>
   <si>
-    <t>UT-031</t>
+    <t>UT-034</t>
   </si>
   <si>
     <t>collects unowned action items into their own group, listed last</t>
@@ -527,7 +569,7 @@
     <t>Total cases</t>
   </si>
   <si>
-    <t>31</t>
+    <t>34</t>
   </si>
   <si>
     <t>Pass criteria</t>
@@ -937,7 +979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1246,39 +1288,39 @@
         <v>56</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="F11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>64</v>
@@ -1287,13 +1329,13 @@
         <v>65</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>67</v>
@@ -1304,10 +1346,10 @@
         <v>68</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>69</v>
@@ -1316,36 +1358,36 @@
         <v>70</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>15</v>
@@ -1354,33 +1396,33 @@
         <v>16</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>80</v>
@@ -1391,10 +1433,10 @@
         <v>81</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>82</v>
@@ -1403,65 +1445,65 @@
         <v>83</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>15</v>
@@ -1470,18 +1512,18 @@
         <v>16</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>95</v>
+        <v>63</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>96</v>
@@ -1490,100 +1532,100 @@
         <v>97</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="G22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>114</v>
@@ -1594,10 +1636,10 @@
         <v>115</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>116</v>
@@ -1606,7 +1648,7 @@
         <v>117</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>15</v>
@@ -1623,48 +1665,48 @@
         <v>119</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>15</v>
@@ -1681,10 +1723,10 @@
         <v>129</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>130</v>
@@ -1693,7 +1735,7 @@
         <v>131</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>15</v>
@@ -1710,10 +1752,10 @@
         <v>133</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>134</v>
@@ -1722,27 +1764,27 @@
         <v>135</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>139</v>
@@ -1751,7 +1793,7 @@
         <v>140</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>15</v>
@@ -1760,27 +1802,27 @@
         <v>16</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="29" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>15</v>
@@ -1789,94 +1831,181 @@
         <v>16</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="F30" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="I30" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="31" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D31" s="2" t="s">
+      <c r="E31" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="F32" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="E32" s="2" t="s">
+    </row>
+    <row r="33" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>161</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -1897,66 +2026,66 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>